<commit_message>
dados: 2026-10-18 08:22 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Jun_2026.xlsx
+++ b/xlsx/carteira_mensal/Jun_2026.xlsx
@@ -174,6 +174,9 @@
     <t>Patricia Souza Fernandez</t>
   </si>
   <si>
+    <t>Já é Cliente</t>
+  </si>
+  <si>
     <t>16/05/26</t>
   </si>
   <si>
@@ -277,9 +280,6 @@
   </si>
   <si>
     <t>Thiago de Souza Silva</t>
-  </si>
-  <si>
-    <t>Já é Cliente</t>
   </si>
   <si>
     <t>26/06/26</t>
@@ -716,25 +716,25 @@
         <v>52</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C32" t="n">
         <v>792.0</v>
       </c>
       <c r="D32" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E32" t="s">
         <v>49</v>
       </c>
       <c r="F32" t="n">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="G32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I32" t="n">
         <v>900.0</v>
@@ -755,12 +755,12 @@
         <v>79202.0</v>
       </c>
       <c r="O32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B33" t="s">
         <v>47</v>
@@ -769,19 +769,19 @@
         <v>819.0</v>
       </c>
       <c r="D33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F33" t="n">
         <v>3.0</v>
       </c>
       <c r="G33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I33" t="n">
         <v>70000.0</v>
@@ -802,24 +802,24 @@
         <v>81902.0</v>
       </c>
       <c r="O33" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B34" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C34" t="n">
         <v>822.0</v>
       </c>
       <c r="D34" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F34" t="n">
         <v>1.0</v>
@@ -828,7 +828,7 @@
         <v>50</v>
       </c>
       <c r="H34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I34" t="n">
         <v>630.0</v>
@@ -849,24 +849,24 @@
         <v>82201.0</v>
       </c>
       <c r="O34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C35" t="n">
         <v>829.0</v>
       </c>
       <c r="D35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F35" t="n">
         <v>1.0</v>
@@ -875,7 +875,7 @@
         <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I35" t="n">
         <v>16800.0</v>
@@ -896,24 +896,24 @@
         <v>82901.0</v>
       </c>
       <c r="O35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C36" t="n">
         <v>832.0</v>
       </c>
       <c r="D36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E36" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
@@ -922,7 +922,7 @@
         <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I36" t="n">
         <v>250000.0</v>
@@ -943,12 +943,12 @@
         <v>83201.0</v>
       </c>
       <c r="O36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
         <v>47</v>
@@ -957,7 +957,7 @@
         <v>830.0</v>
       </c>
       <c r="D37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E37" t="s">
         <v>49</v>
@@ -969,7 +969,7 @@
         <v>50</v>
       </c>
       <c r="H37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I37" t="n">
         <v>12384.22</v>
@@ -990,24 +990,24 @@
         <v>83001.0</v>
       </c>
       <c r="O37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C38" t="n">
         <v>842.0</v>
       </c>
       <c r="D38" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
@@ -1016,7 +1016,7 @@
         <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I38" t="n">
         <v>70000.0</v>
@@ -1037,21 +1037,21 @@
         <v>84201.0</v>
       </c>
       <c r="O38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C39" t="n">
         <v>841.0</v>
       </c>
       <c r="D39" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E39" t="s">
         <v>49</v>
@@ -1060,10 +1060,10 @@
         <v>2.0</v>
       </c>
       <c r="G39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I39" t="n">
         <v>65195.33</v>
@@ -1084,15 +1084,15 @@
         <v>84102.0</v>
       </c>
       <c r="O39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B40" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C40" t="n">
         <v>844.0</v>
@@ -1101,7 +1101,7 @@
         <v>51</v>
       </c>
       <c r="E40" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F40" t="n">
         <v>1.0</v>
@@ -1110,7 +1110,7 @@
         <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I40" t="n">
         <v>9500.0</v>
@@ -1131,12 +1131,12 @@
         <v>84401.0</v>
       </c>
       <c r="O40" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
         <v>47</v>
@@ -1145,10 +1145,10 @@
         <v>846.0</v>
       </c>
       <c r="D41" t="s">
+        <v>60</v>
+      </c>
+      <c r="E41" t="s">
         <v>59</v>
-      </c>
-      <c r="E41" t="s">
-        <v>58</v>
       </c>
       <c r="F41" t="n">
         <v>1.0</v>
@@ -1157,7 +1157,7 @@
         <v>50</v>
       </c>
       <c r="H41" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I41" t="n">
         <v>300.0</v>
@@ -1178,12 +1178,12 @@
         <v>84601.0</v>
       </c>
       <c r="O41" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B42" t="s">
         <v>47</v>
@@ -1192,10 +1192,10 @@
         <v>852.0</v>
       </c>
       <c r="D42" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E42" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F42" t="n">
         <v>1.0</v>
@@ -1204,7 +1204,7 @@
         <v>50</v>
       </c>
       <c r="H42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I42" t="n">
         <v>135000.0</v>
@@ -1225,21 +1225,21 @@
         <v>85201.0</v>
       </c>
       <c r="O42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="C43" t="n">
         <v>857.0</v>
       </c>
       <c r="D43" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E43" t="s">
         <v>49</v>
@@ -1286,7 +1286,7 @@
         <v>856.0</v>
       </c>
       <c r="D44" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E44" t="s">
         <v>91</v>
@@ -1298,7 +1298,7 @@
         <v>50</v>
       </c>
       <c r="H44" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I44" t="n">
         <v>1375.95</v>
@@ -1319,7 +1319,7 @@
         <v>85601.0</v>
       </c>
       <c r="O44" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45">

</xml_diff>